<commit_message>
ALL FN WORKING GOOD
</commit_message>
<xml_diff>
--- a/test/PIPO2_sample.xlsx
+++ b/test/PIPO2_sample.xlsx
@@ -1289,7 +1289,19 @@
   <dimension ref="A1:O5"/>
   <sheetFormatPr defaultColWidth="8.79279279279279" defaultRowHeight="14.4" outlineLevelRow="4"/>
   <cols>
-    <col min="8" max="8" width="11.7927927927928"/>
+    <col min="1" max="1" width="8.78378378378378" customWidth="1"/>
+    <col min="2" max="2" width="15.0810810810811" customWidth="1"/>
+    <col min="3" max="3" width="11.7927927927928" customWidth="1"/>
+    <col min="4" max="4" width="15.963963963964" customWidth="1"/>
+    <col min="5" max="5" width="12.8828828828829" customWidth="1"/>
+    <col min="6" max="6" width="19.6576576576577" customWidth="1"/>
+    <col min="7" max="7" width="15.954954954955" customWidth="1"/>
+    <col min="8" max="8" width="14.1801801801802" customWidth="1"/>
+    <col min="9" max="9" width="16.8918918918919" customWidth="1"/>
+    <col min="10" max="10" width="5.18918918918919" customWidth="1"/>
+    <col min="11" max="11" width="22.6486486486486" customWidth="1"/>
+    <col min="12" max="12" width="21.1711711711712" customWidth="1"/>
+    <col min="13" max="13" width="18.3693693693694" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">

</xml_diff>